<commit_message>
edited new cracmm mechanism info
</commit_message>
<xml_diff>
--- a/F0AM-4.3.0.1/Chem/CB6r5h/CB6r5h_mechanism_info.xlsx
+++ b/F0AM-4.3.0.1/Chem/CB6r5h/CB6r5h_mechanism_info.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanessasun/Documents/phd/utah/research/F0AM_files/final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanessasun/Documents/phd/utah/research/USOS_shared/F0AM-4.3.0.1/Chem/CB6r5h/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07328BD9-4A0B-0E47-ABA2-13F058469EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E01FA04-3234-0A40-A1CA-B22E175A4354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2560" yWindow="960" windowWidth="22520" windowHeight="20780" activeTab="1" xr2:uid="{8D81D372-274D-BA44-8D8F-526417B0CB6D}"/>
+    <workbookView xWindow="8680" yWindow="1300" windowWidth="28080" windowHeight="20780" activeTab="3" xr2:uid="{8D81D372-274D-BA44-8D8F-526417B0CB6D}"/>
   </bookViews>
   <sheets>
     <sheet name="k rate" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1866" uniqueCount="1008">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1867" uniqueCount="1009">
   <si>
     <t>Reaction</t>
   </si>
@@ -3066,6 +3066,9 @@
   </si>
   <si>
     <t>InChI=1S/C3H8/c1-3-2/h3H2,1-2H3</t>
+  </si>
+  <si>
+    <t>acryloyl peroxynitrate</t>
   </si>
 </sst>
 </file>
@@ -8892,6 +8895,9 @@
         <f>_xlfn.XLOOKUP(A57,mech1!B$2:B$121,mech1!A$2:A$121,"")</f>
         <v/>
       </c>
+      <c r="F57" t="s">
+        <v>1008</v>
+      </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="15" t="s">

</xml_diff>

<commit_message>
New USOS campaign plots, started looking at EPA VOC preliminary data
</commit_message>
<xml_diff>
--- a/F0AM-4.3.0.1/Chem/CB6r5h/CB6r5h_mechanism_info.xlsx
+++ b/F0AM-4.3.0.1/Chem/CB6r5h/CB6r5h_mechanism_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanessasun/Documents/phd/utah/research/USOS_shared/F0AM-4.3.0.1/Chem/CB6r5h/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E01FA04-3234-0A40-A1CA-B22E175A4354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E2B825-5D03-2A46-91BC-15CD56758297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8680" yWindow="1300" windowWidth="28080" windowHeight="20780" activeTab="3" xr2:uid="{8D81D372-274D-BA44-8D8F-526417B0CB6D}"/>
+    <workbookView xWindow="21100" yWindow="500" windowWidth="17620" windowHeight="20780" activeTab="1" xr2:uid="{8D81D372-274D-BA44-8D8F-526417B0CB6D}"/>
   </bookViews>
   <sheets>
     <sheet name="k rate" sheetId="1" r:id="rId1"/>

</xml_diff>